<commit_message>
modified llm output result
</commit_message>
<xml_diff>
--- a/llm-summarize-document/output_rag/summaries.xlsx
+++ b/llm-summarize-document/output_rag/summaries.xlsx
@@ -1,37 +1,63 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+  <si>
+    <t>Filename</t>
+  </si>
+  <si>
+    <t>Summary</t>
+  </si>
+  <si>
+    <t>langchain_demo.txt</t>
+  </si>
+  <si>
+    <t>sample.pdf</t>
+  </si>
+  <si>
+    <t>LangChain is a framework designed to simplify the development of LLM-powered applications. It offers modular components, data integration, agent frameworks, memory management, and prompt engineering tools, enabling developers to build applications like chatbots, question answering systems, summarization tools, and autonomous agents. The document encourages users to explore the official documentation and YouTube channel for further learning and resources.</t>
+  </si>
+  <si>
+    <t>This document is a placeholder text sample ("Lorem Ipsum") used for design mockups and testing. It contains a collection of Latin phrases and placeholder text commonly used in the graphic design industry.</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
   <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -46,93 +72,35 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
 </file>
 
@@ -420,51 +388,35 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Filename</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Summary</t>
-        </is>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>langchain_demo.txt</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>LangChain is a framework designed to simplify the building of LLM-powered applications. Its key features involve modular components, seamless data integration, agent frameworks, memory management, prompt engineering, and chain optimization, enabling a wide range of applications like chatbots, question answering systems, and text generation tools. Resources like documentation and a YouTube channel by Brandon Hancock are available for further learning.</t>
-        </is>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>sample.pdf</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>This document is a placeholder text (Lorem Ipsum) – a standard dummy text used in design and printing to demonstrate the visual form of a document without relying on meaningful content.</t>
-        </is>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>